<commit_message>
Update function Xuất Kho
</commit_message>
<xml_diff>
--- a/MPR_Managerment/Templates/pxk_template.xlsx
+++ b/MPR_Managerment/Templates/pxk_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RÁC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ERP_Final_Management\MPR_Managerment\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F8A5062E-6E4B-4706-82BF-EEF54445A7BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34FD528C-68C1-43FB-BA48-CEB22733DF8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C76654CC-9D16-46A5-BBB8-C0EB8C5DB89A}"/>
+    <workbookView xWindow="-28920" yWindow="735" windowWidth="29040" windowHeight="15720" xr2:uid="{C76654CC-9D16-46A5-BBB8-C0EB8C5DB89A}"/>
   </bookViews>
   <sheets>
     <sheet name="PXK" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="31">
   <si>
     <t>MATERIAL REQUISTION FORM
 MẪU YÊU CẦU VẬT TƯ</t>
@@ -43,20 +43,72 @@
     <t>Effective Date:</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Job No </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <i/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(Mã dự án)</t>
-    </r>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Description (Diễn giải)</t>
+  </si>
+  <si>
+    <t>Q’ty</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>Remark</t>
+  </si>
+  <si>
+    <t>Code
+(Mã số VL)</t>
+  </si>
+  <si>
+    <t>Name
+(Tên)</t>
+  </si>
+  <si>
+    <t>DWG No
+(Bản vẽ số)</t>
+  </si>
+  <si>
+    <t>Size
+(Kích thước)</t>
+  </si>
+  <si>
+    <t>Grade/ Class
+(Cấp độ / Loại)</t>
+  </si>
+  <si>
+    <t>(Số lượng)</t>
+  </si>
+  <si>
+    <t>(Đơn vị tính)</t>
+  </si>
+  <si>
+    <t>(Ghi chú)</t>
+  </si>
+  <si>
+    <t>Prepared by Foreman</t>
+  </si>
+  <si>
+    <t>Approved by Production Eng./ Manager</t>
+  </si>
+  <si>
+    <t>Approved by Planning Management</t>
+  </si>
+  <si>
+    <t>Issued by Material Control</t>
+  </si>
+  <si>
+    <t>&lt;&lt;SUM&gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;DATE&gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;PROJECT-NAME&gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;USER&gt;&gt;</t>
   </si>
   <si>
     <r>
@@ -67,10 +119,26 @@
         <i/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
       </rPr>
       <t>(Số phát hành):</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Job No </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(Mã dự án)</t>
     </r>
   </si>
   <si>
@@ -81,10 +149,10 @@
       <rPr>
         <b/>
         <i/>
-        <sz val="10"/>
+        <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
       </rPr>
       <t>(Tên dự án)</t>
     </r>
@@ -96,10 +164,10 @@
     <r>
       <rPr>
         <i/>
-        <sz val="10"/>
+        <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
       </rPr>
       <t>(Người nhận):</t>
     </r>
@@ -112,10 +180,10 @@
       <rPr>
         <b/>
         <i/>
-        <sz val="10"/>
+        <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
       </rPr>
       <t>(Số sản phẩm)</t>
     </r>
@@ -127,82 +195,20 @@
     <r>
       <rPr>
         <i/>
-        <sz val="10"/>
+        <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
       </rPr>
       <t>(Ngày):</t>
     </r>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Description (Diễn giải)</t>
-  </si>
-  <si>
-    <t>Q’ty</t>
-  </si>
-  <si>
-    <t>Unit</t>
-  </si>
-  <si>
-    <t>Remark</t>
-  </si>
-  <si>
-    <t>Code
-(Mã số VL)</t>
-  </si>
-  <si>
-    <t>Name
-(Tên)</t>
-  </si>
-  <si>
-    <t>DWG No
-(Bản vẽ số)</t>
-  </si>
-  <si>
-    <t>Size
-(Kích thước)</t>
-  </si>
-  <si>
-    <t>Grade/ Class
-(Cấp độ / Loại)</t>
-  </si>
-  <si>
-    <t>(Số lượng)</t>
-  </si>
-  <si>
-    <t>(Đơn vị tính)</t>
-  </si>
-  <si>
-    <t>(Ghi chú)</t>
-  </si>
-  <si>
-    <t>Prepared by Foreman</t>
-  </si>
-  <si>
-    <t>Approved by Production Eng./ Manager</t>
-  </si>
-  <si>
-    <t>Approved by Planning Management</t>
-  </si>
-  <si>
-    <t>Issued by Material Control</t>
-  </si>
-  <si>
-    <t>&lt;&lt;SUM&gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt;DATE&gt;&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -211,123 +217,86 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="18"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <i/>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
       <i/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -410,115 +379,112 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="15" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="15" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -919,234 +885,252 @@
   <dimension ref="A2:M15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.42578125" style="4" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" style="4" customWidth="1"/>
-    <col min="3" max="3" width="28" style="4" customWidth="1"/>
-    <col min="4" max="4" width="21" style="4" customWidth="1"/>
-    <col min="5" max="5" width="25.140625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="16.85546875" style="4" customWidth="1"/>
-    <col min="7" max="7" width="14.5703125" style="4" customWidth="1"/>
-    <col min="8" max="8" width="14.140625" style="4" customWidth="1"/>
-    <col min="9" max="9" width="22.7109375" style="4" customWidth="1"/>
-    <col min="10" max="10" width="9.140625" style="4"/>
-    <col min="11" max="11" width="15.7109375" style="4" customWidth="1"/>
-    <col min="12" max="12" width="9.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.28515625" style="4" customWidth="1"/>
-    <col min="14" max="16384" width="9.140625" style="4"/>
+    <col min="1" max="1" width="6.42578125" style="5" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="28" style="5" customWidth="1"/>
+    <col min="4" max="4" width="21" style="5" customWidth="1"/>
+    <col min="5" max="5" width="25.140625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="16.85546875" style="5" customWidth="1"/>
+    <col min="7" max="7" width="14.5703125" style="5" customWidth="1"/>
+    <col min="8" max="8" width="14.140625" style="5" customWidth="1"/>
+    <col min="9" max="9" width="22.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="9.140625" style="5"/>
+    <col min="11" max="11" width="15.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="9.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.28515625" style="5" customWidth="1"/>
+    <col min="14" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="2" t="s">
+      <c r="A2" s="31"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="3" t="s">
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="3"/>
+      <c r="I2" s="4"/>
     </row>
     <row r="3" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="3" t="s">
+      <c r="A3" s="31"/>
+      <c r="B3" s="31"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I3" s="3"/>
+      <c r="I3" s="4"/>
     </row>
     <row r="4" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="3" t="s">
+      <c r="A4" s="31"/>
+      <c r="B4" s="31"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32"/>
+      <c r="G4" s="32"/>
+      <c r="H4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="5"/>
+      <c r="I4" s="6"/>
     </row>
     <row r="5" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="6"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="8"/>
-      <c r="I5" s="9"/>
+      <c r="A5" s="7"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="10"/>
     </row>
     <row r="6" spans="1:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="35"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" s="27"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="30"/>
+    </row>
+    <row r="7" spans="1:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="35"/>
+      <c r="C7" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="25"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="27" t="s">
+        <v>28</v>
+      </c>
+      <c r="G7" s="27" t="s">
+        <v>28</v>
+      </c>
+      <c r="H7" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="I7" s="28"/>
+    </row>
+    <row r="8" spans="1:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="35" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="35"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="27" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" s="27" t="s">
+        <v>30</v>
+      </c>
+      <c r="H8" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="I8" s="28"/>
+    </row>
+    <row r="9" spans="1:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="10"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="14" t="s">
+      <c r="B9" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="14"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
-    </row>
-    <row r="7" spans="1:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="10"/>
-      <c r="C7" s="16"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="14" t="s">
+      <c r="H9" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="G7" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
-    </row>
-    <row r="8" spans="1:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+      <c r="I9" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="14" t="s">
+    </row>
+    <row r="10" spans="1:13" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="22"/>
+      <c r="B10" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="H8" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="I8" s="17"/>
-    </row>
-    <row r="9" spans="1:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
+      <c r="C10" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="20" t="s">
+      <c r="D10" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="21" t="s">
+      <c r="E10" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="H9" s="21" t="s">
+      <c r="F10" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="I9" s="21" t="s">
+      <c r="G10" s="15" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="19"/>
-      <c r="B10" s="21" t="s">
+      <c r="H10" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="21" t="s">
+      <c r="I10" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="D10" s="21" t="s">
+    </row>
+    <row r="11" spans="1:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="12"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="34"/>
+      <c r="G11" s="34"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="34"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="3"/>
+      <c r="M11" s="3"/>
+    </row>
+    <row r="12" spans="1:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="1"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="H12" s="14"/>
+      <c r="I12" s="17"/>
+      <c r="K12" s="18"/>
+    </row>
+    <row r="14" spans="1:13" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="E10" s="21" t="s">
+      <c r="B14" s="23"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="21" t="s">
+      <c r="E14" s="23"/>
+      <c r="F14" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="G10" s="22" t="s">
+      <c r="G14" s="23"/>
+      <c r="H14" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="H10" s="22" t="s">
-        <v>21</v>
-      </c>
-      <c r="I10" s="22" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="23"/>
-      <c r="B11" s="21"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="24"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="24"/>
-      <c r="H11" s="21"/>
-      <c r="I11" s="24"/>
-      <c r="J11" s="35"/>
-      <c r="K11" s="36"/>
-      <c r="L11" s="36"/>
-      <c r="M11" s="36"/>
-    </row>
-    <row r="12" spans="1:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="23"/>
-      <c r="B12" s="25"/>
-      <c r="C12" s="21"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="28"/>
-      <c r="G12" s="21" t="s">
-        <v>27</v>
-      </c>
-      <c r="H12" s="21"/>
-      <c r="I12" s="29"/>
-      <c r="K12" s="30"/>
-    </row>
-    <row r="14" spans="1:13" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="31" t="s">
-        <v>23</v>
-      </c>
-      <c r="B14" s="31"/>
-      <c r="C14" s="31"/>
-      <c r="D14" s="31" t="s">
-        <v>24</v>
-      </c>
-      <c r="E14" s="31"/>
-      <c r="F14" s="31" t="s">
-        <v>25</v>
-      </c>
-      <c r="G14" s="31"/>
-      <c r="H14" s="31" t="s">
-        <v>26</v>
-      </c>
-      <c r="I14" s="31"/>
+      <c r="I14" s="23"/>
     </row>
     <row r="15" spans="1:13" ht="93" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="32"/>
-      <c r="B15" s="33"/>
-      <c r="C15" s="34"/>
-      <c r="D15" s="32"/>
-      <c r="E15" s="34"/>
-      <c r="F15" s="32"/>
-      <c r="G15" s="34"/>
-      <c r="H15" s="32"/>
-      <c r="I15" s="34"/>
+      <c r="A15" s="19"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="21"/>
+      <c r="H15" s="19"/>
+      <c r="I15" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="A2:B4"/>
+    <mergeCell ref="C2:G4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:E7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:E8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="H8:I8"/>
     <mergeCell ref="A15:C15"/>
     <mergeCell ref="D15:E15"/>
     <mergeCell ref="F15:G15"/>
@@ -1157,20 +1141,6 @@
     <mergeCell ref="D14:E14"/>
     <mergeCell ref="F14:G14"/>
     <mergeCell ref="H14:I14"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:E7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C8:E8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="A2:B4"/>
-    <mergeCell ref="C2:G4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:E6"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="H6:I6"/>
   </mergeCells>
   <conditionalFormatting sqref="C11 E11:E12">
     <cfRule type="expression" dxfId="2" priority="1">

</xml_diff>

<commit_message>
Update tạo phiếu yêu cầu xuất vật tư
</commit_message>
<xml_diff>
--- a/MPR_Managerment/Templates/pxk_template.xlsx
+++ b/MPR_Managerment/Templates/pxk_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ERP_Final_Management\MPR_Managerment\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34FD528C-68C1-43FB-BA48-CEB22733DF8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9965F449-4D57-4EA9-AA56-15741B45E3B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="735" windowWidth="29040" windowHeight="15720" xr2:uid="{C76654CC-9D16-46A5-BBB8-C0EB8C5DB89A}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="PXK" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">PXK!$A$1:$I$15</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">PXK!$A$1:$J$15</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="32">
   <si>
     <t>MATERIAL REQUISTION FORM
 MẪU YÊU CẦU VẬT TƯ</t>
@@ -202,6 +202,9 @@
       </rPr>
       <t>(Ngày):</t>
     </r>
+  </si>
+  <si>
+    <t>ID_Code</t>
   </si>
 </sst>
 </file>
@@ -435,6 +438,42 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -449,42 +488,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -882,7 +885,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:M15"/>
+  <dimension ref="A2:N15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.42578125" style="5" customWidth="1"/>
@@ -892,57 +895,60 @@
     <col min="5" max="5" width="25.140625" style="5" customWidth="1"/>
     <col min="6" max="6" width="16.85546875" style="5" customWidth="1"/>
     <col min="7" max="7" width="14.5703125" style="5" customWidth="1"/>
-    <col min="8" max="8" width="14.140625" style="5" customWidth="1"/>
-    <col min="9" max="9" width="22.7109375" style="5" customWidth="1"/>
-    <col min="10" max="10" width="9.140625" style="5"/>
-    <col min="11" max="11" width="15.7109375" style="5" customWidth="1"/>
-    <col min="12" max="12" width="9.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.28515625" style="5" customWidth="1"/>
-    <col min="14" max="16384" width="9.140625" style="5"/>
+    <col min="8" max="9" width="14.140625" style="5" customWidth="1"/>
+    <col min="10" max="10" width="22.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="9.140625" style="5"/>
+    <col min="12" max="12" width="15.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="9.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.28515625" style="5" customWidth="1"/>
+    <col min="15" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="31"/>
-      <c r="B2" s="31"/>
-      <c r="C2" s="32" t="s">
+    <row r="2" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="21"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
       <c r="H2" s="4" t="s">
         <v>1</v>
       </c>
       <c r="I2" s="4"/>
-    </row>
-    <row r="3" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="31"/>
-      <c r="B3" s="31"/>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
+      <c r="J2" s="4"/>
+    </row>
+    <row r="3" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="21"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
       <c r="H3" s="4" t="s">
         <v>2</v>
       </c>
       <c r="I3" s="4"/>
-    </row>
-    <row r="4" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="31"/>
-      <c r="B4" s="31"/>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
-      <c r="F4" s="32"/>
-      <c r="G4" s="32"/>
+      <c r="J3" s="4"/>
+    </row>
+    <row r="4" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="21"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
       <c r="H4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="6"/>
-    </row>
-    <row r="5" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I4" s="4"/>
+      <c r="J4" s="6"/>
+    </row>
+    <row r="5" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -951,29 +957,31 @@
       <c r="F5" s="8"/>
       <c r="G5" s="8"/>
       <c r="H5" s="9"/>
-      <c r="I5" s="10"/>
-    </row>
-    <row r="6" spans="1:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="35" t="s">
+      <c r="I5" s="9"/>
+      <c r="J5" s="10"/>
+    </row>
+    <row r="6" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="35"/>
-      <c r="C6" s="33"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="24"/>
       <c r="D6" s="25"/>
       <c r="E6" s="26"/>
       <c r="F6" s="27" t="s">
         <v>25</v>
       </c>
       <c r="G6" s="27"/>
-      <c r="H6" s="30"/>
-      <c r="I6" s="30"/>
-    </row>
-    <row r="7" spans="1:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="35" t="s">
+      <c r="H6" s="20"/>
+      <c r="I6" s="20"/>
+      <c r="J6" s="20"/>
+    </row>
+    <row r="7" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="35"/>
-      <c r="C7" s="24" t="s">
+      <c r="B7" s="23"/>
+      <c r="C7" s="28" t="s">
         <v>23</v>
       </c>
       <c r="D7" s="25"/>
@@ -984,17 +992,18 @@
       <c r="G7" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="H7" s="28" t="s">
+      <c r="H7" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="I7" s="28"/>
-    </row>
-    <row r="8" spans="1:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="35" t="s">
+      <c r="I7" s="29"/>
+      <c r="J7" s="29"/>
+    </row>
+    <row r="8" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="B8" s="35"/>
-      <c r="C8" s="24"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="28"/>
       <c r="D8" s="25"/>
       <c r="E8" s="26"/>
       <c r="F8" s="27" t="s">
@@ -1003,22 +1012,23 @@
       <c r="G8" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="29" t="s">
+      <c r="H8" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="I8" s="28"/>
-    </row>
-    <row r="9" spans="1:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="22" t="s">
+      <c r="I8" s="30"/>
+      <c r="J8" s="29"/>
+    </row>
+    <row r="9" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="22"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="22"/>
-      <c r="F9" s="22"/>
+      <c r="C9" s="34"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="34"/>
+      <c r="F9" s="34"/>
       <c r="G9" s="14" t="s">
         <v>6</v>
       </c>
@@ -1026,11 +1036,14 @@
         <v>7</v>
       </c>
       <c r="I9" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="J9" s="14" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="22"/>
+    <row r="10" spans="1:14" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="34"/>
       <c r="B10" s="14" t="s">
         <v>9</v>
       </c>
@@ -1053,25 +1066,29 @@
         <v>15</v>
       </c>
       <c r="I10" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="J10" s="15" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="12"/>
       <c r="B11" s="11"/>
-      <c r="C11" s="34"/>
-      <c r="D11" s="34"/>
-      <c r="E11" s="34"/>
-      <c r="F11" s="34"/>
-      <c r="G11" s="34"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
       <c r="H11" s="11"/>
-      <c r="I11" s="34"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="3"/>
+      <c r="I11" s="11"/>
+      <c r="J11" s="19"/>
+      <c r="K11" s="2"/>
       <c r="L11" s="3"/>
       <c r="M11" s="3"/>
-    </row>
-    <row r="12" spans="1:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N11" s="3"/>
+    </row>
+    <row r="12" spans="1:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="13"/>
       <c r="C12" s="14"/>
@@ -1082,65 +1099,68 @@
         <v>21</v>
       </c>
       <c r="H12" s="14"/>
-      <c r="I12" s="17"/>
-      <c r="K12" s="18"/>
-    </row>
-    <row r="14" spans="1:13" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="23" t="s">
+      <c r="I12" s="14"/>
+      <c r="J12" s="17"/>
+      <c r="L12" s="18"/>
+    </row>
+    <row r="14" spans="1:14" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="23"/>
-      <c r="C14" s="23"/>
-      <c r="D14" s="23" t="s">
+      <c r="B14" s="35"/>
+      <c r="C14" s="35"/>
+      <c r="D14" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23" t="s">
+      <c r="E14" s="35"/>
+      <c r="F14" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="G14" s="23"/>
-      <c r="H14" s="23" t="s">
+      <c r="G14" s="35"/>
+      <c r="H14" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="I14" s="23"/>
-    </row>
-    <row r="15" spans="1:13" ht="93" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="19"/>
-      <c r="B15" s="20"/>
-      <c r="C15" s="21"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="21"/>
-      <c r="H15" s="19"/>
-      <c r="I15" s="21"/>
+      <c r="I14" s="35"/>
+      <c r="J14" s="35"/>
+    </row>
+    <row r="15" spans="1:14" ht="93" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="31"/>
+      <c r="B15" s="32"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="33"/>
+      <c r="F15" s="31"/>
+      <c r="G15" s="33"/>
+      <c r="H15" s="31"/>
+      <c r="I15" s="32"/>
+      <c r="J15" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:E7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:E8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="H6:J6"/>
     <mergeCell ref="A2:B4"/>
     <mergeCell ref="C2:G4"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:E6"/>
     <mergeCell ref="F6:G6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:E7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C8:E8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="H15:I15"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="H14:I14"/>
   </mergeCells>
   <conditionalFormatting sqref="C11 E11:E12">
     <cfRule type="expression" dxfId="2" priority="1">

</xml_diff>